<commit_message>
Handle rank column, improve parse_file
</commit_message>
<xml_diff>
--- a/tests/data/test_file.xlsx
+++ b/tests/data/test_file.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
   <si>
     <t xml:space="preserve">Réponse</t>
   </si>
@@ -43,6 +43,9 @@
     <t xml:space="preserve">ID</t>
   </si>
   <si>
+    <t xml:space="preserve">Classement</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nom complet</t>
   </si>
   <si>
@@ -103,6 +106,9 @@
     <t xml:space="preserve">ADS :  voeux</t>
   </si>
   <si>
+    <t xml:space="preserve">aze</t>
+  </si>
+  <si>
     <t xml:space="preserve">Laurence Marchand</t>
   </si>
   <si>
@@ -115,6 +121,9 @@
     <t xml:space="preserve">{INRIA}03</t>
   </si>
   <si>
+    <t xml:space="preserve">ert</t>
+  </si>
+  <si>
     <t xml:space="preserve">Laurence ROZE</t>
   </si>
   <si>
@@ -125,6 +134,9 @@
   </si>
   <si>
     <t xml:space="preserve">{EES}0350936C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yui</t>
   </si>
   <si>
     <t xml:space="preserve">Laurence Roze</t>
@@ -171,7 +183,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -221,11 +232,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -352,7 +363,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:AA4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -380,56 +391,60 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="1"/>
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>24</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -440,16 +455,16 @@
         <v>45587.6108796296</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>5747</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>27</v>
+      <c r="H2" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>28</v>
@@ -457,29 +472,35 @@
       <c r="J2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="K2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="L2" s="1" t="n">
+      <c r="N2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="M2" s="1" t="n">
+      <c r="O2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="N2" s="1" t="n">
+      <c r="P2" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="O2" s="1" t="n">
+      <c r="Q2" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="P2" s="1" t="n">
+      <c r="R2" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="Q2" s="1" t="n">
+      <c r="S2" s="1" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>15076</v>
       </c>
@@ -487,33 +508,39 @@
         <v>45587.6222453704</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>17639</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>31</v>
+      <c r="H3" s="1" t="n">
+        <v>2</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="R3" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="T3" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="S3" s="1" t="n">
+      <c r="U3" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="T3" s="1" t="n">
+      <c r="V3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="U3" s="1" t="n">
+      <c r="W3" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -525,33 +552,39 @@
         <v>45587.6244212963</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>17640</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>35</v>
+      <c r="H4" s="1" t="n">
+        <v>3</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V4" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X4" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="W4" s="1" t="n">
+      <c r="Y4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="X4" s="1" t="n">
+      <c r="Z4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="Y4" s="1" t="n">
+      <c r="AA4" s="1" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>